<commit_message>
Update README and login test evidence
</commit_message>
<xml_diff>
--- a/test-cases/login-test-cases.xlsx
+++ b/test-cases/login-test-cases.xlsx
@@ -877,7 +877,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="9">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -892,9 +892,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -1453,25 +1450,25 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" spans="1:7">
-      <c r="A1" s="6" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="B1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="6" t="s">
+      <c r="C1" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="6" t="s">
+      <c r="D1" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="6" t="s">
+      <c r="E1" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="6" t="s">
+      <c r="F1" s="5" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="6" t="s">
+      <c r="G1" s="5" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1494,7 +1491,7 @@
       <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="7" t="s">
+      <c r="G2" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1517,7 +1514,7 @@
       <c r="F3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="G3" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1540,7 +1537,7 @@
       <c r="F4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="7" t="s">
+      <c r="G4" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1563,7 +1560,7 @@
       <c r="F5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="G5" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1586,7 +1583,7 @@
       <c r="F6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="7" t="s">
+      <c r="G6" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1609,7 +1606,7 @@
       <c r="F7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="7" t="s">
+      <c r="G7" s="6" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1632,396 +1629,396 @@
       <c r="F8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="7" t="s">
+      <c r="G8" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="8"/>
-      <c r="B9" s="8"/>
-      <c r="C9" s="8"/>
-      <c r="D9" s="8"/>
-      <c r="E9" s="8"/>
-      <c r="F9" s="8"/>
-      <c r="G9" s="8"/>
+      <c r="A9" s="7"/>
+      <c r="B9" s="7"/>
+      <c r="C9" s="7"/>
+      <c r="D9" s="7"/>
+      <c r="E9" s="7"/>
+      <c r="F9" s="7"/>
+      <c r="G9" s="7"/>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="8"/>
-      <c r="B10" s="8"/>
-      <c r="C10" s="8"/>
-      <c r="D10" s="8"/>
-      <c r="E10" s="8"/>
-      <c r="F10" s="8"/>
-      <c r="G10" s="8"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="7"/>
+      <c r="C10" s="7"/>
+      <c r="D10" s="7"/>
+      <c r="E10" s="7"/>
+      <c r="F10" s="7"/>
+      <c r="G10" s="7"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="8"/>
-      <c r="B11" s="8"/>
-      <c r="C11" s="8"/>
-      <c r="D11" s="8"/>
-      <c r="E11" s="8"/>
-      <c r="F11" s="8"/>
-      <c r="G11" s="8"/>
+      <c r="A11" s="7"/>
+      <c r="B11" s="7"/>
+      <c r="C11" s="7"/>
+      <c r="D11" s="7"/>
+      <c r="E11" s="7"/>
+      <c r="F11" s="7"/>
+      <c r="G11" s="7"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="8"/>
-      <c r="B12" s="8"/>
-      <c r="C12" s="8"/>
-      <c r="D12" s="8"/>
-      <c r="E12" s="8"/>
-      <c r="F12" s="8"/>
-      <c r="G12" s="8"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="7"/>
+      <c r="C12" s="7"/>
+      <c r="D12" s="7"/>
+      <c r="E12" s="7"/>
+      <c r="F12" s="7"/>
+      <c r="G12" s="7"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="8"/>
-      <c r="B13" s="8"/>
-      <c r="C13" s="8"/>
-      <c r="D13" s="8"/>
-      <c r="E13" s="8"/>
-      <c r="F13" s="8"/>
-      <c r="G13" s="8"/>
+      <c r="A13" s="7"/>
+      <c r="B13" s="7"/>
+      <c r="C13" s="7"/>
+      <c r="D13" s="7"/>
+      <c r="E13" s="7"/>
+      <c r="F13" s="7"/>
+      <c r="G13" s="7"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="8"/>
-      <c r="B14" s="8"/>
-      <c r="C14" s="8"/>
-      <c r="D14" s="8"/>
-      <c r="E14" s="8"/>
-      <c r="F14" s="8"/>
-      <c r="G14" s="8"/>
+      <c r="A14" s="7"/>
+      <c r="B14" s="7"/>
+      <c r="C14" s="7"/>
+      <c r="D14" s="7"/>
+      <c r="E14" s="7"/>
+      <c r="F14" s="7"/>
+      <c r="G14" s="7"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="8"/>
-      <c r="B15" s="8"/>
-      <c r="C15" s="8"/>
-      <c r="D15" s="8"/>
-      <c r="E15" s="8"/>
-      <c r="F15" s="8"/>
-      <c r="G15" s="8"/>
+      <c r="A15" s="7"/>
+      <c r="B15" s="7"/>
+      <c r="C15" s="7"/>
+      <c r="D15" s="7"/>
+      <c r="E15" s="7"/>
+      <c r="F15" s="7"/>
+      <c r="G15" s="7"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="8"/>
-      <c r="B16" s="8"/>
-      <c r="C16" s="8"/>
-      <c r="D16" s="8"/>
-      <c r="E16" s="8"/>
-      <c r="F16" s="8"/>
-      <c r="G16" s="8"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="7"/>
+      <c r="C16" s="7"/>
+      <c r="D16" s="7"/>
+      <c r="E16" s="7"/>
+      <c r="F16" s="7"/>
+      <c r="G16" s="7"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="8"/>
-      <c r="B17" s="8"/>
-      <c r="C17" s="8"/>
-      <c r="D17" s="8"/>
-      <c r="E17" s="8"/>
-      <c r="F17" s="8"/>
-      <c r="G17" s="8"/>
+      <c r="A17" s="7"/>
+      <c r="B17" s="7"/>
+      <c r="C17" s="7"/>
+      <c r="D17" s="7"/>
+      <c r="E17" s="7"/>
+      <c r="F17" s="7"/>
+      <c r="G17" s="7"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="8"/>
-      <c r="B18" s="8"/>
-      <c r="C18" s="8"/>
-      <c r="D18" s="8"/>
-      <c r="E18" s="8"/>
-      <c r="F18" s="8"/>
-      <c r="G18" s="8"/>
+      <c r="A18" s="7"/>
+      <c r="B18" s="7"/>
+      <c r="C18" s="7"/>
+      <c r="D18" s="7"/>
+      <c r="E18" s="7"/>
+      <c r="F18" s="7"/>
+      <c r="G18" s="7"/>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="8"/>
-      <c r="B19" s="8"/>
-      <c r="C19" s="8"/>
-      <c r="D19" s="8"/>
-      <c r="E19" s="8"/>
-      <c r="F19" s="8"/>
-      <c r="G19" s="8"/>
+      <c r="A19" s="7"/>
+      <c r="B19" s="7"/>
+      <c r="C19" s="7"/>
+      <c r="D19" s="7"/>
+      <c r="E19" s="7"/>
+      <c r="F19" s="7"/>
+      <c r="G19" s="7"/>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="8"/>
-      <c r="B20" s="8"/>
-      <c r="C20" s="8"/>
-      <c r="D20" s="8"/>
-      <c r="E20" s="8"/>
-      <c r="F20" s="8"/>
-      <c r="G20" s="8"/>
+      <c r="A20" s="7"/>
+      <c r="B20" s="7"/>
+      <c r="C20" s="7"/>
+      <c r="D20" s="7"/>
+      <c r="E20" s="7"/>
+      <c r="F20" s="7"/>
+      <c r="G20" s="7"/>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="8"/>
-      <c r="B21" s="8"/>
-      <c r="C21" s="8"/>
-      <c r="D21" s="8"/>
-      <c r="E21" s="8"/>
-      <c r="F21" s="8"/>
-      <c r="G21" s="8"/>
+      <c r="A21" s="7"/>
+      <c r="B21" s="7"/>
+      <c r="C21" s="7"/>
+      <c r="D21" s="7"/>
+      <c r="E21" s="7"/>
+      <c r="F21" s="7"/>
+      <c r="G21" s="7"/>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="8"/>
-      <c r="B22" s="8"/>
-      <c r="C22" s="8"/>
-      <c r="D22" s="8"/>
-      <c r="E22" s="8"/>
-      <c r="F22" s="8"/>
-      <c r="G22" s="8"/>
+      <c r="A22" s="7"/>
+      <c r="B22" s="7"/>
+      <c r="C22" s="7"/>
+      <c r="D22" s="7"/>
+      <c r="E22" s="7"/>
+      <c r="F22" s="7"/>
+      <c r="G22" s="7"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="8"/>
-      <c r="B23" s="8"/>
-      <c r="C23" s="8"/>
-      <c r="D23" s="8"/>
-      <c r="E23" s="9"/>
-      <c r="F23" s="8"/>
-      <c r="G23" s="8"/>
+      <c r="A23" s="7"/>
+      <c r="B23" s="7"/>
+      <c r="C23" s="7"/>
+      <c r="D23" s="7"/>
+      <c r="E23" s="8"/>
+      <c r="F23" s="7"/>
+      <c r="G23" s="7"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="8"/>
-      <c r="B24" s="8"/>
-      <c r="C24" s="8"/>
-      <c r="D24" s="8"/>
-      <c r="E24" s="8"/>
-      <c r="F24" s="8"/>
-      <c r="G24" s="8"/>
+      <c r="A24" s="7"/>
+      <c r="B24" s="7"/>
+      <c r="C24" s="7"/>
+      <c r="D24" s="7"/>
+      <c r="E24" s="7"/>
+      <c r="F24" s="7"/>
+      <c r="G24" s="7"/>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="8"/>
-      <c r="B25" s="8"/>
-      <c r="C25" s="8"/>
-      <c r="D25" s="8"/>
-      <c r="E25" s="8"/>
-      <c r="F25" s="8"/>
-      <c r="G25" s="8"/>
+      <c r="A25" s="7"/>
+      <c r="B25" s="7"/>
+      <c r="C25" s="7"/>
+      <c r="D25" s="7"/>
+      <c r="E25" s="7"/>
+      <c r="F25" s="7"/>
+      <c r="G25" s="7"/>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="8"/>
-      <c r="B26" s="8"/>
-      <c r="C26" s="8"/>
-      <c r="D26" s="8"/>
-      <c r="E26" s="8"/>
-      <c r="F26" s="8"/>
-      <c r="G26" s="8"/>
+      <c r="A26" s="7"/>
+      <c r="B26" s="7"/>
+      <c r="C26" s="7"/>
+      <c r="D26" s="7"/>
+      <c r="E26" s="7"/>
+      <c r="F26" s="7"/>
+      <c r="G26" s="7"/>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="8"/>
-      <c r="B27" s="8"/>
-      <c r="C27" s="8"/>
-      <c r="D27" s="8"/>
-      <c r="E27" s="8"/>
-      <c r="F27" s="8"/>
-      <c r="G27" s="8"/>
+      <c r="A27" s="7"/>
+      <c r="B27" s="7"/>
+      <c r="C27" s="7"/>
+      <c r="D27" s="7"/>
+      <c r="E27" s="7"/>
+      <c r="F27" s="7"/>
+      <c r="G27" s="7"/>
     </row>
     <row r="28" spans="1:7">
-      <c r="A28" s="8"/>
-      <c r="B28" s="8"/>
-      <c r="C28" s="8"/>
-      <c r="D28" s="8"/>
-      <c r="E28" s="8"/>
-      <c r="F28" s="8"/>
-      <c r="G28" s="8"/>
+      <c r="A28" s="7"/>
+      <c r="B28" s="7"/>
+      <c r="C28" s="7"/>
+      <c r="D28" s="7"/>
+      <c r="E28" s="7"/>
+      <c r="F28" s="7"/>
+      <c r="G28" s="7"/>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="8"/>
-      <c r="B29" s="8"/>
-      <c r="C29" s="8"/>
-      <c r="D29" s="8"/>
-      <c r="E29" s="8"/>
-      <c r="F29" s="8"/>
-      <c r="G29" s="8"/>
+      <c r="A29" s="7"/>
+      <c r="B29" s="7"/>
+      <c r="C29" s="7"/>
+      <c r="D29" s="7"/>
+      <c r="E29" s="7"/>
+      <c r="F29" s="7"/>
+      <c r="G29" s="7"/>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="8"/>
-      <c r="B30" s="8"/>
-      <c r="C30" s="8"/>
-      <c r="D30" s="8"/>
-      <c r="E30" s="8"/>
-      <c r="F30" s="8"/>
-      <c r="G30" s="8"/>
+      <c r="A30" s="7"/>
+      <c r="B30" s="7"/>
+      <c r="C30" s="7"/>
+      <c r="D30" s="7"/>
+      <c r="E30" s="7"/>
+      <c r="F30" s="7"/>
+      <c r="G30" s="7"/>
     </row>
     <row r="31" spans="1:7">
-      <c r="A31" s="8"/>
-      <c r="B31" s="8"/>
-      <c r="C31" s="8"/>
-      <c r="D31" s="8"/>
-      <c r="E31" s="8"/>
-      <c r="F31" s="8"/>
-      <c r="G31" s="8"/>
+      <c r="A31" s="7"/>
+      <c r="B31" s="7"/>
+      <c r="C31" s="7"/>
+      <c r="D31" s="7"/>
+      <c r="E31" s="7"/>
+      <c r="F31" s="7"/>
+      <c r="G31" s="7"/>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="8"/>
-      <c r="B32" s="8"/>
-      <c r="C32" s="8"/>
-      <c r="D32" s="8"/>
-      <c r="E32" s="8"/>
-      <c r="F32" s="8"/>
-      <c r="G32" s="8"/>
+      <c r="A32" s="7"/>
+      <c r="B32" s="7"/>
+      <c r="C32" s="7"/>
+      <c r="D32" s="7"/>
+      <c r="E32" s="7"/>
+      <c r="F32" s="7"/>
+      <c r="G32" s="7"/>
     </row>
     <row r="33" spans="1:7">
-      <c r="A33" s="8"/>
-      <c r="B33" s="8"/>
-      <c r="C33" s="8"/>
-      <c r="D33" s="8"/>
-      <c r="E33" s="8"/>
-      <c r="F33" s="8"/>
-      <c r="G33" s="8"/>
+      <c r="A33" s="7"/>
+      <c r="B33" s="7"/>
+      <c r="C33" s="7"/>
+      <c r="D33" s="7"/>
+      <c r="E33" s="7"/>
+      <c r="F33" s="7"/>
+      <c r="G33" s="7"/>
     </row>
     <row r="34" spans="1:7">
-      <c r="A34" s="8"/>
-      <c r="B34" s="8"/>
-      <c r="C34" s="8"/>
-      <c r="D34" s="8"/>
-      <c r="E34" s="8"/>
-      <c r="F34" s="8"/>
-      <c r="G34" s="8"/>
+      <c r="A34" s="7"/>
+      <c r="B34" s="7"/>
+      <c r="C34" s="7"/>
+      <c r="D34" s="7"/>
+      <c r="E34" s="7"/>
+      <c r="F34" s="7"/>
+      <c r="G34" s="7"/>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="8"/>
-      <c r="B35" s="8"/>
-      <c r="C35" s="8"/>
-      <c r="D35" s="8"/>
-      <c r="E35" s="8"/>
-      <c r="F35" s="8"/>
-      <c r="G35" s="8"/>
+      <c r="A35" s="7"/>
+      <c r="B35" s="7"/>
+      <c r="C35" s="7"/>
+      <c r="D35" s="7"/>
+      <c r="E35" s="7"/>
+      <c r="F35" s="7"/>
+      <c r="G35" s="7"/>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="8"/>
-      <c r="B36" s="8"/>
-      <c r="C36" s="8"/>
-      <c r="D36" s="8"/>
-      <c r="E36" s="8"/>
-      <c r="F36" s="8"/>
-      <c r="G36" s="8"/>
+      <c r="A36" s="7"/>
+      <c r="B36" s="7"/>
+      <c r="C36" s="7"/>
+      <c r="D36" s="7"/>
+      <c r="E36" s="7"/>
+      <c r="F36" s="7"/>
+      <c r="G36" s="7"/>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="8"/>
-      <c r="B37" s="8"/>
-      <c r="C37" s="8"/>
-      <c r="D37" s="8"/>
-      <c r="E37" s="8"/>
-      <c r="F37" s="8"/>
-      <c r="G37" s="8"/>
+      <c r="A37" s="7"/>
+      <c r="B37" s="7"/>
+      <c r="C37" s="7"/>
+      <c r="D37" s="7"/>
+      <c r="E37" s="7"/>
+      <c r="F37" s="7"/>
+      <c r="G37" s="7"/>
     </row>
     <row r="38" spans="1:7">
-      <c r="A38" s="8"/>
-      <c r="B38" s="8"/>
-      <c r="C38" s="8"/>
-      <c r="D38" s="8"/>
-      <c r="E38" s="8"/>
-      <c r="F38" s="8"/>
-      <c r="G38" s="8"/>
+      <c r="A38" s="7"/>
+      <c r="B38" s="7"/>
+      <c r="C38" s="7"/>
+      <c r="D38" s="7"/>
+      <c r="E38" s="7"/>
+      <c r="F38" s="7"/>
+      <c r="G38" s="7"/>
     </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="8"/>
-      <c r="B39" s="8"/>
-      <c r="C39" s="8"/>
-      <c r="D39" s="8"/>
-      <c r="E39" s="8"/>
-      <c r="F39" s="8"/>
-      <c r="G39" s="8"/>
+      <c r="A39" s="7"/>
+      <c r="B39" s="7"/>
+      <c r="C39" s="7"/>
+      <c r="D39" s="7"/>
+      <c r="E39" s="7"/>
+      <c r="F39" s="7"/>
+      <c r="G39" s="7"/>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="8"/>
-      <c r="B40" s="8"/>
-      <c r="C40" s="8"/>
-      <c r="D40" s="8"/>
-      <c r="E40" s="8"/>
-      <c r="F40" s="8"/>
-      <c r="G40" s="8"/>
+      <c r="A40" s="7"/>
+      <c r="B40" s="7"/>
+      <c r="C40" s="7"/>
+      <c r="D40" s="7"/>
+      <c r="E40" s="7"/>
+      <c r="F40" s="7"/>
+      <c r="G40" s="7"/>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="8"/>
-      <c r="B41" s="8"/>
-      <c r="C41" s="8"/>
-      <c r="D41" s="8"/>
-      <c r="E41" s="8"/>
-      <c r="F41" s="8"/>
-      <c r="G41" s="8"/>
+      <c r="A41" s="7"/>
+      <c r="B41" s="7"/>
+      <c r="C41" s="7"/>
+      <c r="D41" s="7"/>
+      <c r="E41" s="7"/>
+      <c r="F41" s="7"/>
+      <c r="G41" s="7"/>
     </row>
     <row r="42" spans="1:7">
-      <c r="A42" s="8"/>
-      <c r="B42" s="8"/>
-      <c r="C42" s="8"/>
-      <c r="D42" s="8"/>
-      <c r="E42" s="8"/>
-      <c r="F42" s="8"/>
-      <c r="G42" s="8"/>
+      <c r="A42" s="7"/>
+      <c r="B42" s="7"/>
+      <c r="C42" s="7"/>
+      <c r="D42" s="7"/>
+      <c r="E42" s="7"/>
+      <c r="F42" s="7"/>
+      <c r="G42" s="7"/>
     </row>
     <row r="43" spans="1:7">
-      <c r="A43" s="8"/>
-      <c r="B43" s="8"/>
-      <c r="C43" s="8"/>
-      <c r="D43" s="8"/>
-      <c r="E43" s="8"/>
-      <c r="F43" s="8"/>
-      <c r="G43" s="8"/>
+      <c r="A43" s="7"/>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7"/>
+      <c r="D43" s="7"/>
+      <c r="E43" s="7"/>
+      <c r="F43" s="7"/>
+      <c r="G43" s="7"/>
     </row>
     <row r="44" spans="1:7">
-      <c r="A44" s="8"/>
-      <c r="B44" s="8"/>
-      <c r="C44" s="8"/>
-      <c r="D44" s="8"/>
-      <c r="E44" s="8"/>
-      <c r="F44" s="8"/>
-      <c r="G44" s="8"/>
+      <c r="A44" s="7"/>
+      <c r="B44" s="7"/>
+      <c r="C44" s="7"/>
+      <c r="D44" s="7"/>
+      <c r="E44" s="7"/>
+      <c r="F44" s="7"/>
+      <c r="G44" s="7"/>
     </row>
     <row r="45" spans="1:7">
-      <c r="A45" s="8"/>
-      <c r="B45" s="8"/>
-      <c r="C45" s="8"/>
-      <c r="D45" s="8"/>
-      <c r="E45" s="8"/>
-      <c r="F45" s="8"/>
-      <c r="G45" s="8"/>
+      <c r="A45" s="7"/>
+      <c r="B45" s="7"/>
+      <c r="C45" s="7"/>
+      <c r="D45" s="7"/>
+      <c r="E45" s="7"/>
+      <c r="F45" s="7"/>
+      <c r="G45" s="7"/>
     </row>
     <row r="46" spans="1:7">
-      <c r="A46" s="8"/>
-      <c r="B46" s="8"/>
-      <c r="C46" s="8"/>
-      <c r="D46" s="8"/>
-      <c r="E46" s="8"/>
-      <c r="F46" s="8"/>
-      <c r="G46" s="8"/>
+      <c r="A46" s="7"/>
+      <c r="B46" s="7"/>
+      <c r="C46" s="7"/>
+      <c r="D46" s="7"/>
+      <c r="E46" s="7"/>
+      <c r="F46" s="7"/>
+      <c r="G46" s="7"/>
     </row>
     <row r="47" spans="1:7">
-      <c r="A47" s="8"/>
-      <c r="B47" s="8"/>
-      <c r="C47" s="8"/>
-      <c r="D47" s="8"/>
-      <c r="E47" s="8"/>
-      <c r="F47" s="8"/>
-      <c r="G47" s="8"/>
+      <c r="A47" s="7"/>
+      <c r="B47" s="7"/>
+      <c r="C47" s="7"/>
+      <c r="D47" s="7"/>
+      <c r="E47" s="7"/>
+      <c r="F47" s="7"/>
+      <c r="G47" s="7"/>
     </row>
     <row r="48" spans="1:7">
-      <c r="A48" s="8"/>
-      <c r="B48" s="8"/>
-      <c r="C48" s="8"/>
-      <c r="D48" s="8"/>
-      <c r="E48" s="8"/>
-      <c r="F48" s="8"/>
-      <c r="G48" s="8"/>
+      <c r="A48" s="7"/>
+      <c r="B48" s="7"/>
+      <c r="C48" s="7"/>
+      <c r="D48" s="7"/>
+      <c r="E48" s="7"/>
+      <c r="F48" s="7"/>
+      <c r="G48" s="7"/>
     </row>
     <row r="49" spans="1:7">
-      <c r="A49" s="8"/>
-      <c r="B49" s="8"/>
-      <c r="C49" s="8"/>
-      <c r="D49" s="8"/>
-      <c r="E49" s="8"/>
-      <c r="F49" s="8"/>
-      <c r="G49" s="8"/>
+      <c r="A49" s="7"/>
+      <c r="B49" s="7"/>
+      <c r="C49" s="7"/>
+      <c r="D49" s="7"/>
+      <c r="E49" s="7"/>
+      <c r="F49" s="7"/>
+      <c r="G49" s="7"/>
     </row>
     <row r="50" spans="1:7">
-      <c r="A50" s="8"/>
-      <c r="B50" s="8"/>
-      <c r="C50" s="8"/>
-      <c r="D50" s="8"/>
-      <c r="E50" s="8"/>
-      <c r="F50" s="8"/>
-      <c r="G50" s="8"/>
+      <c r="A50" s="7"/>
+      <c r="B50" s="7"/>
+      <c r="C50" s="7"/>
+      <c r="D50" s="7"/>
+      <c r="E50" s="7"/>
+      <c r="F50" s="7"/>
+      <c r="G50" s="7"/>
     </row>
     <row r="51" spans="1:7">
-      <c r="A51" s="8"/>
-      <c r="B51" s="8"/>
-      <c r="C51" s="8"/>
-      <c r="D51" s="8"/>
-      <c r="E51" s="8"/>
-      <c r="F51" s="8"/>
-      <c r="G51" s="8"/>
+      <c r="A51" s="7"/>
+      <c r="B51" s="7"/>
+      <c r="C51" s="7"/>
+      <c r="D51" s="7"/>
+      <c r="E51" s="7"/>
+      <c r="F51" s="7"/>
+      <c r="G51" s="7"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2099,7 +2096,7 @@
       <c r="F3" s="2"/>
     </row>
     <row r="4" ht="44" customHeight="1" spans="1:6">
-      <c r="A4" s="5" t="s">
+      <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
       <c r="B4" s="3" t="s">
@@ -2147,7 +2144,7 @@
       <c r="F6" s="2"/>
     </row>
     <row r="7" ht="74" customHeight="1" spans="1:6">
-      <c r="A7" s="5" t="s">
+      <c r="A7" s="2" t="s">
         <v>33</v>
       </c>
       <c r="B7" s="3" t="s">
@@ -2163,7 +2160,7 @@
       <c r="F7" s="2"/>
     </row>
     <row r="8" ht="42.75" spans="1:6">
-      <c r="A8" s="5" t="s">
+      <c r="A8" s="2" t="s">
         <v>39</v>
       </c>
       <c r="B8" s="3" t="s">

</xml_diff>

<commit_message>
Add product listing test cases and evidence
</commit_message>
<xml_diff>
--- a/test-cases/login-test-cases.xlsx
+++ b/test-cases/login-test-cases.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="17580"/>
+    <workbookView windowHeight="17580" activeTab="1"/>
   </bookViews>
   <sheets>
     <sheet name="Test Cases" sheetId="2" r:id="rId1"/>
@@ -253,11 +253,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="xr9">
-  <numFmts count="4">
+  <numFmts count="5">
     <numFmt numFmtId="176" formatCode="_-* #,##0.00_-;\-* #,##0.00_-;_-* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="177" formatCode="_-&quot;฿&quot;* #,##0.00_-;\-&quot;฿&quot;* #,##0.00_-;_-&quot;฿&quot;* &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="178" formatCode="_-* #,##0_-;\-* #,##0_-;_-* &quot;-&quot;_-;_-@_-"/>
     <numFmt numFmtId="179" formatCode="_-&quot;฿&quot;* #,##0_-;\-&quot;฿&quot;* #,##0_-;_-&quot;฿&quot;* &quot;-&quot;_-;_-@_-"/>
+    <numFmt numFmtId="180" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="20">
     <font>
@@ -877,7 +878,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -891,6 +892,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="180" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -1450,25 +1454,25 @@
   </cols>
   <sheetData>
     <row r="1" ht="15.75" spans="1:7">
-      <c r="A1" s="5" t="s">
+      <c r="A1" s="6" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5" t="s">
+      <c r="B1" s="6" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="5" t="s">
+      <c r="C1" s="6" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="5" t="s">
+      <c r="D1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="5" t="s">
+      <c r="E1" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="5" t="s">
+      <c r="F1" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="5" t="s">
+      <c r="G1" s="6" t="s">
         <v>6</v>
       </c>
     </row>
@@ -1491,7 +1495,7 @@
       <c r="F2" s="3" t="s">
         <v>12</v>
       </c>
-      <c r="G2" s="6" t="s">
+      <c r="G2" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1514,7 +1518,7 @@
       <c r="F3" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G3" s="6" t="s">
+      <c r="G3" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1537,7 +1541,7 @@
       <c r="F4" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G4" s="6" t="s">
+      <c r="G4" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1560,7 +1564,7 @@
       <c r="F5" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G5" s="6" t="s">
+      <c r="G5" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1583,7 +1587,7 @@
       <c r="F6" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="G6" s="6" t="s">
+      <c r="G6" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1606,7 +1610,7 @@
       <c r="F7" s="3" t="s">
         <v>38</v>
       </c>
-      <c r="G7" s="6" t="s">
+      <c r="G7" s="7" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1629,396 +1633,396 @@
       <c r="F8" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G8" s="6" t="s">
+      <c r="G8" s="7" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:7">
-      <c r="A9" s="7"/>
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-      <c r="F9" s="7"/>
-      <c r="G9" s="7"/>
+      <c r="A9" s="8"/>
+      <c r="B9" s="8"/>
+      <c r="C9" s="8"/>
+      <c r="D9" s="8"/>
+      <c r="E9" s="8"/>
+      <c r="F9" s="8"/>
+      <c r="G9" s="8"/>
     </row>
     <row r="10" spans="1:7">
-      <c r="A10" s="7"/>
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-      <c r="F10" s="7"/>
-      <c r="G10" s="7"/>
+      <c r="A10" s="8"/>
+      <c r="B10" s="8"/>
+      <c r="C10" s="8"/>
+      <c r="D10" s="8"/>
+      <c r="E10" s="8"/>
+      <c r="F10" s="8"/>
+      <c r="G10" s="8"/>
     </row>
     <row r="11" spans="1:7">
-      <c r="A11" s="7"/>
-      <c r="B11" s="7"/>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-      <c r="F11" s="7"/>
-      <c r="G11" s="7"/>
+      <c r="A11" s="8"/>
+      <c r="B11" s="8"/>
+      <c r="C11" s="8"/>
+      <c r="D11" s="8"/>
+      <c r="E11" s="8"/>
+      <c r="F11" s="8"/>
+      <c r="G11" s="8"/>
     </row>
     <row r="12" spans="1:7">
-      <c r="A12" s="7"/>
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7"/>
-      <c r="G12" s="7"/>
+      <c r="A12" s="8"/>
+      <c r="B12" s="8"/>
+      <c r="C12" s="8"/>
+      <c r="D12" s="8"/>
+      <c r="E12" s="8"/>
+      <c r="F12" s="8"/>
+      <c r="G12" s="8"/>
     </row>
     <row r="13" spans="1:7">
-      <c r="A13" s="7"/>
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
-      <c r="G13" s="7"/>
+      <c r="A13" s="8"/>
+      <c r="B13" s="8"/>
+      <c r="C13" s="8"/>
+      <c r="D13" s="8"/>
+      <c r="E13" s="8"/>
+      <c r="F13" s="8"/>
+      <c r="G13" s="8"/>
     </row>
     <row r="14" spans="1:7">
-      <c r="A14" s="7"/>
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
-      <c r="G14" s="7"/>
+      <c r="A14" s="8"/>
+      <c r="B14" s="8"/>
+      <c r="C14" s="8"/>
+      <c r="D14" s="8"/>
+      <c r="E14" s="8"/>
+      <c r="F14" s="8"/>
+      <c r="G14" s="8"/>
     </row>
     <row r="15" spans="1:7">
-      <c r="A15" s="7"/>
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
-      <c r="G15" s="7"/>
+      <c r="A15" s="8"/>
+      <c r="B15" s="8"/>
+      <c r="C15" s="8"/>
+      <c r="D15" s="8"/>
+      <c r="E15" s="8"/>
+      <c r="F15" s="8"/>
+      <c r="G15" s="8"/>
     </row>
     <row r="16" spans="1:7">
-      <c r="A16" s="7"/>
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
-      <c r="G16" s="7"/>
+      <c r="A16" s="8"/>
+      <c r="B16" s="8"/>
+      <c r="C16" s="8"/>
+      <c r="D16" s="8"/>
+      <c r="E16" s="8"/>
+      <c r="F16" s="8"/>
+      <c r="G16" s="8"/>
     </row>
     <row r="17" spans="1:7">
-      <c r="A17" s="7"/>
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
-      <c r="G17" s="7"/>
+      <c r="A17" s="8"/>
+      <c r="B17" s="8"/>
+      <c r="C17" s="8"/>
+      <c r="D17" s="8"/>
+      <c r="E17" s="8"/>
+      <c r="F17" s="8"/>
+      <c r="G17" s="8"/>
     </row>
     <row r="18" spans="1:7">
-      <c r="A18" s="7"/>
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
-      <c r="G18" s="7"/>
+      <c r="A18" s="8"/>
+      <c r="B18" s="8"/>
+      <c r="C18" s="8"/>
+      <c r="D18" s="8"/>
+      <c r="E18" s="8"/>
+      <c r="F18" s="8"/>
+      <c r="G18" s="8"/>
     </row>
     <row r="19" spans="1:7">
-      <c r="A19" s="7"/>
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
-      <c r="G19" s="7"/>
+      <c r="A19" s="8"/>
+      <c r="B19" s="8"/>
+      <c r="C19" s="8"/>
+      <c r="D19" s="8"/>
+      <c r="E19" s="8"/>
+      <c r="F19" s="8"/>
+      <c r="G19" s="8"/>
     </row>
     <row r="20" spans="1:7">
-      <c r="A20" s="7"/>
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
-      <c r="G20" s="7"/>
+      <c r="A20" s="8"/>
+      <c r="B20" s="8"/>
+      <c r="C20" s="8"/>
+      <c r="D20" s="8"/>
+      <c r="E20" s="8"/>
+      <c r="F20" s="8"/>
+      <c r="G20" s="8"/>
     </row>
     <row r="21" spans="1:7">
-      <c r="A21" s="7"/>
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-      <c r="F21" s="7"/>
-      <c r="G21" s="7"/>
+      <c r="A21" s="8"/>
+      <c r="B21" s="8"/>
+      <c r="C21" s="8"/>
+      <c r="D21" s="8"/>
+      <c r="E21" s="8"/>
+      <c r="F21" s="8"/>
+      <c r="G21" s="8"/>
     </row>
     <row r="22" spans="1:7">
-      <c r="A22" s="7"/>
-      <c r="B22" s="7"/>
-      <c r="C22" s="7"/>
-      <c r="D22" s="7"/>
-      <c r="E22" s="7"/>
-      <c r="F22" s="7"/>
-      <c r="G22" s="7"/>
+      <c r="A22" s="8"/>
+      <c r="B22" s="8"/>
+      <c r="C22" s="8"/>
+      <c r="D22" s="8"/>
+      <c r="E22" s="8"/>
+      <c r="F22" s="8"/>
+      <c r="G22" s="8"/>
     </row>
     <row r="23" spans="1:7">
-      <c r="A23" s="7"/>
-      <c r="B23" s="7"/>
-      <c r="C23" s="7"/>
-      <c r="D23" s="7"/>
-      <c r="E23" s="8"/>
-      <c r="F23" s="7"/>
-      <c r="G23" s="7"/>
+      <c r="A23" s="8"/>
+      <c r="B23" s="8"/>
+      <c r="C23" s="8"/>
+      <c r="D23" s="8"/>
+      <c r="E23" s="9"/>
+      <c r="F23" s="8"/>
+      <c r="G23" s="8"/>
     </row>
     <row r="24" spans="1:7">
-      <c r="A24" s="7"/>
-      <c r="B24" s="7"/>
-      <c r="C24" s="7"/>
-      <c r="D24" s="7"/>
-      <c r="E24" s="7"/>
-      <c r="F24" s="7"/>
-      <c r="G24" s="7"/>
+      <c r="A24" s="8"/>
+      <c r="B24" s="8"/>
+      <c r="C24" s="8"/>
+      <c r="D24" s="8"/>
+      <c r="E24" s="8"/>
+      <c r="F24" s="8"/>
+      <c r="G24" s="8"/>
     </row>
     <row r="25" spans="1:7">
-      <c r="A25" s="7"/>
-      <c r="B25" s="7"/>
-      <c r="C25" s="7"/>
-      <c r="D25" s="7"/>
-      <c r="E25" s="7"/>
-      <c r="F25" s="7"/>
-      <c r="G25" s="7"/>
+      <c r="A25" s="8"/>
+      <c r="B25" s="8"/>
+      <c r="C25" s="8"/>
+      <c r="D25" s="8"/>
+      <c r="E25" s="8"/>
+      <c r="F25" s="8"/>
+      <c r="G25" s="8"/>
     </row>
     <row r="26" spans="1:7">
-      <c r="A26" s="7"/>
-      <c r="B26" s="7"/>
-      <c r="C26" s="7"/>
-      <c r="D26" s="7"/>
-      <c r="E26" s="7"/>
-      <c r="F26" s="7"/>
-      <c r="G26" s="7"/>
+      <c r="A26" s="8"/>
+      <c r="B26" s="8"/>
+      <c r="C26" s="8"/>
+      <c r="D26" s="8"/>
+      <c r="E26" s="8"/>
+      <c r="F26" s="8"/>
+      <c r="G26" s="8"/>
     </row>
     <row r="27" spans="1:7">
-      <c r="A27" s="7"/>
-      <c r="B27" s="7"/>
-      <c r="C27" s="7"/>
-      <c r="D27" s="7"/>
-      <c r="E27" s="7"/>
-      <c r="F27" s="7"/>
-      <c r="G27" s="7"/>
+      <c r="A27" s="8"/>
+      <c r="B27" s="8"/>
+      <c r="C27" s="8"/>
+      <c r="D27" s="8"/>
+      <c r="E27" s="8"/>
+      <c r="F27" s="8"/>
+      <c r="G27" s="8"/>
     </row>
     <row r="28" spans="1:7">
-      <c r="A28" s="7"/>
-      <c r="B28" s="7"/>
-      <c r="C28" s="7"/>
-      <c r="D28" s="7"/>
-      <c r="E28" s="7"/>
-      <c r="F28" s="7"/>
-      <c r="G28" s="7"/>
+      <c r="A28" s="8"/>
+      <c r="B28" s="8"/>
+      <c r="C28" s="8"/>
+      <c r="D28" s="8"/>
+      <c r="E28" s="8"/>
+      <c r="F28" s="8"/>
+      <c r="G28" s="8"/>
     </row>
     <row r="29" spans="1:7">
-      <c r="A29" s="7"/>
-      <c r="B29" s="7"/>
-      <c r="C29" s="7"/>
-      <c r="D29" s="7"/>
-      <c r="E29" s="7"/>
-      <c r="F29" s="7"/>
-      <c r="G29" s="7"/>
+      <c r="A29" s="8"/>
+      <c r="B29" s="8"/>
+      <c r="C29" s="8"/>
+      <c r="D29" s="8"/>
+      <c r="E29" s="8"/>
+      <c r="F29" s="8"/>
+      <c r="G29" s="8"/>
     </row>
     <row r="30" spans="1:7">
-      <c r="A30" s="7"/>
-      <c r="B30" s="7"/>
-      <c r="C30" s="7"/>
-      <c r="D30" s="7"/>
-      <c r="E30" s="7"/>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
+      <c r="A30" s="8"/>
+      <c r="B30" s="8"/>
+      <c r="C30" s="8"/>
+      <c r="D30" s="8"/>
+      <c r="E30" s="8"/>
+      <c r="F30" s="8"/>
+      <c r="G30" s="8"/>
     </row>
     <row r="31" spans="1:7">
-      <c r="A31" s="7"/>
-      <c r="B31" s="7"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
+      <c r="A31" s="8"/>
+      <c r="B31" s="8"/>
+      <c r="C31" s="8"/>
+      <c r="D31" s="8"/>
+      <c r="E31" s="8"/>
+      <c r="F31" s="8"/>
+      <c r="G31" s="8"/>
     </row>
     <row r="32" spans="1:7">
-      <c r="A32" s="7"/>
-      <c r="B32" s="7"/>
-      <c r="C32" s="7"/>
-      <c r="D32" s="7"/>
-      <c r="E32" s="7"/>
-      <c r="F32" s="7"/>
-      <c r="G32" s="7"/>
+      <c r="A32" s="8"/>
+      <c r="B32" s="8"/>
+      <c r="C32" s="8"/>
+      <c r="D32" s="8"/>
+      <c r="E32" s="8"/>
+      <c r="F32" s="8"/>
+      <c r="G32" s="8"/>
     </row>
     <row r="33" spans="1:7">
-      <c r="A33" s="7"/>
-      <c r="B33" s="7"/>
-      <c r="C33" s="7"/>
-      <c r="D33" s="7"/>
-      <c r="E33" s="7"/>
-      <c r="F33" s="7"/>
-      <c r="G33" s="7"/>
+      <c r="A33" s="8"/>
+      <c r="B33" s="8"/>
+      <c r="C33" s="8"/>
+      <c r="D33" s="8"/>
+      <c r="E33" s="8"/>
+      <c r="F33" s="8"/>
+      <c r="G33" s="8"/>
     </row>
     <row r="34" spans="1:7">
-      <c r="A34" s="7"/>
-      <c r="B34" s="7"/>
-      <c r="C34" s="7"/>
-      <c r="D34" s="7"/>
-      <c r="E34" s="7"/>
-      <c r="F34" s="7"/>
-      <c r="G34" s="7"/>
+      <c r="A34" s="8"/>
+      <c r="B34" s="8"/>
+      <c r="C34" s="8"/>
+      <c r="D34" s="8"/>
+      <c r="E34" s="8"/>
+      <c r="F34" s="8"/>
+      <c r="G34" s="8"/>
     </row>
     <row r="35" spans="1:7">
-      <c r="A35" s="7"/>
-      <c r="B35" s="7"/>
-      <c r="C35" s="7"/>
-      <c r="D35" s="7"/>
-      <c r="E35" s="7"/>
-      <c r="F35" s="7"/>
-      <c r="G35" s="7"/>
+      <c r="A35" s="8"/>
+      <c r="B35" s="8"/>
+      <c r="C35" s="8"/>
+      <c r="D35" s="8"/>
+      <c r="E35" s="8"/>
+      <c r="F35" s="8"/>
+      <c r="G35" s="8"/>
     </row>
     <row r="36" spans="1:7">
-      <c r="A36" s="7"/>
-      <c r="B36" s="7"/>
-      <c r="C36" s="7"/>
-      <c r="D36" s="7"/>
-      <c r="E36" s="7"/>
-      <c r="F36" s="7"/>
-      <c r="G36" s="7"/>
+      <c r="A36" s="8"/>
+      <c r="B36" s="8"/>
+      <c r="C36" s="8"/>
+      <c r="D36" s="8"/>
+      <c r="E36" s="8"/>
+      <c r="F36" s="8"/>
+      <c r="G36" s="8"/>
     </row>
     <row r="37" spans="1:7">
-      <c r="A37" s="7"/>
-      <c r="B37" s="7"/>
-      <c r="C37" s="7"/>
-      <c r="D37" s="7"/>
-      <c r="E37" s="7"/>
-      <c r="F37" s="7"/>
-      <c r="G37" s="7"/>
+      <c r="A37" s="8"/>
+      <c r="B37" s="8"/>
+      <c r="C37" s="8"/>
+      <c r="D37" s="8"/>
+      <c r="E37" s="8"/>
+      <c r="F37" s="8"/>
+      <c r="G37" s="8"/>
     </row>
     <row r="38" spans="1:7">
-      <c r="A38" s="7"/>
-      <c r="B38" s="7"/>
-      <c r="C38" s="7"/>
-      <c r="D38" s="7"/>
-      <c r="E38" s="7"/>
-      <c r="F38" s="7"/>
-      <c r="G38" s="7"/>
+      <c r="A38" s="8"/>
+      <c r="B38" s="8"/>
+      <c r="C38" s="8"/>
+      <c r="D38" s="8"/>
+      <c r="E38" s="8"/>
+      <c r="F38" s="8"/>
+      <c r="G38" s="8"/>
     </row>
     <row r="39" spans="1:7">
-      <c r="A39" s="7"/>
-      <c r="B39" s="7"/>
-      <c r="C39" s="7"/>
-      <c r="D39" s="7"/>
-      <c r="E39" s="7"/>
-      <c r="F39" s="7"/>
-      <c r="G39" s="7"/>
+      <c r="A39" s="8"/>
+      <c r="B39" s="8"/>
+      <c r="C39" s="8"/>
+      <c r="D39" s="8"/>
+      <c r="E39" s="8"/>
+      <c r="F39" s="8"/>
+      <c r="G39" s="8"/>
     </row>
     <row r="40" spans="1:7">
-      <c r="A40" s="7"/>
-      <c r="B40" s="7"/>
-      <c r="C40" s="7"/>
-      <c r="D40" s="7"/>
-      <c r="E40" s="7"/>
-      <c r="F40" s="7"/>
-      <c r="G40" s="7"/>
+      <c r="A40" s="8"/>
+      <c r="B40" s="8"/>
+      <c r="C40" s="8"/>
+      <c r="D40" s="8"/>
+      <c r="E40" s="8"/>
+      <c r="F40" s="8"/>
+      <c r="G40" s="8"/>
     </row>
     <row r="41" spans="1:7">
-      <c r="A41" s="7"/>
-      <c r="B41" s="7"/>
-      <c r="C41" s="7"/>
-      <c r="D41" s="7"/>
-      <c r="E41" s="7"/>
-      <c r="F41" s="7"/>
-      <c r="G41" s="7"/>
+      <c r="A41" s="8"/>
+      <c r="B41" s="8"/>
+      <c r="C41" s="8"/>
+      <c r="D41" s="8"/>
+      <c r="E41" s="8"/>
+      <c r="F41" s="8"/>
+      <c r="G41" s="8"/>
     </row>
     <row r="42" spans="1:7">
-      <c r="A42" s="7"/>
-      <c r="B42" s="7"/>
-      <c r="C42" s="7"/>
-      <c r="D42" s="7"/>
-      <c r="E42" s="7"/>
-      <c r="F42" s="7"/>
-      <c r="G42" s="7"/>
+      <c r="A42" s="8"/>
+      <c r="B42" s="8"/>
+      <c r="C42" s="8"/>
+      <c r="D42" s="8"/>
+      <c r="E42" s="8"/>
+      <c r="F42" s="8"/>
+      <c r="G42" s="8"/>
     </row>
     <row r="43" spans="1:7">
-      <c r="A43" s="7"/>
-      <c r="B43" s="7"/>
-      <c r="C43" s="7"/>
-      <c r="D43" s="7"/>
-      <c r="E43" s="7"/>
-      <c r="F43" s="7"/>
-      <c r="G43" s="7"/>
+      <c r="A43" s="8"/>
+      <c r="B43" s="8"/>
+      <c r="C43" s="8"/>
+      <c r="D43" s="8"/>
+      <c r="E43" s="8"/>
+      <c r="F43" s="8"/>
+      <c r="G43" s="8"/>
     </row>
     <row r="44" spans="1:7">
-      <c r="A44" s="7"/>
-      <c r="B44" s="7"/>
-      <c r="C44" s="7"/>
-      <c r="D44" s="7"/>
-      <c r="E44" s="7"/>
-      <c r="F44" s="7"/>
-      <c r="G44" s="7"/>
+      <c r="A44" s="8"/>
+      <c r="B44" s="8"/>
+      <c r="C44" s="8"/>
+      <c r="D44" s="8"/>
+      <c r="E44" s="8"/>
+      <c r="F44" s="8"/>
+      <c r="G44" s="8"/>
     </row>
     <row r="45" spans="1:7">
-      <c r="A45" s="7"/>
-      <c r="B45" s="7"/>
-      <c r="C45" s="7"/>
-      <c r="D45" s="7"/>
-      <c r="E45" s="7"/>
-      <c r="F45" s="7"/>
-      <c r="G45" s="7"/>
+      <c r="A45" s="8"/>
+      <c r="B45" s="8"/>
+      <c r="C45" s="8"/>
+      <c r="D45" s="8"/>
+      <c r="E45" s="8"/>
+      <c r="F45" s="8"/>
+      <c r="G45" s="8"/>
     </row>
     <row r="46" spans="1:7">
-      <c r="A46" s="7"/>
-      <c r="B46" s="7"/>
-      <c r="C46" s="7"/>
-      <c r="D46" s="7"/>
-      <c r="E46" s="7"/>
-      <c r="F46" s="7"/>
-      <c r="G46" s="7"/>
+      <c r="A46" s="8"/>
+      <c r="B46" s="8"/>
+      <c r="C46" s="8"/>
+      <c r="D46" s="8"/>
+      <c r="E46" s="8"/>
+      <c r="F46" s="8"/>
+      <c r="G46" s="8"/>
     </row>
     <row r="47" spans="1:7">
-      <c r="A47" s="7"/>
-      <c r="B47" s="7"/>
-      <c r="C47" s="7"/>
-      <c r="D47" s="7"/>
-      <c r="E47" s="7"/>
-      <c r="F47" s="7"/>
-      <c r="G47" s="7"/>
+      <c r="A47" s="8"/>
+      <c r="B47" s="8"/>
+      <c r="C47" s="8"/>
+      <c r="D47" s="8"/>
+      <c r="E47" s="8"/>
+      <c r="F47" s="8"/>
+      <c r="G47" s="8"/>
     </row>
     <row r="48" spans="1:7">
-      <c r="A48" s="7"/>
-      <c r="B48" s="7"/>
-      <c r="C48" s="7"/>
-      <c r="D48" s="7"/>
-      <c r="E48" s="7"/>
-      <c r="F48" s="7"/>
-      <c r="G48" s="7"/>
+      <c r="A48" s="8"/>
+      <c r="B48" s="8"/>
+      <c r="C48" s="8"/>
+      <c r="D48" s="8"/>
+      <c r="E48" s="8"/>
+      <c r="F48" s="8"/>
+      <c r="G48" s="8"/>
     </row>
     <row r="49" spans="1:7">
-      <c r="A49" s="7"/>
-      <c r="B49" s="7"/>
-      <c r="C49" s="7"/>
-      <c r="D49" s="7"/>
-      <c r="E49" s="7"/>
-      <c r="F49" s="7"/>
-      <c r="G49" s="7"/>
+      <c r="A49" s="8"/>
+      <c r="B49" s="8"/>
+      <c r="C49" s="8"/>
+      <c r="D49" s="8"/>
+      <c r="E49" s="8"/>
+      <c r="F49" s="8"/>
+      <c r="G49" s="8"/>
     </row>
     <row r="50" spans="1:7">
-      <c r="A50" s="7"/>
-      <c r="B50" s="7"/>
-      <c r="C50" s="7"/>
-      <c r="D50" s="7"/>
-      <c r="E50" s="7"/>
-      <c r="F50" s="7"/>
-      <c r="G50" s="7"/>
+      <c r="A50" s="8"/>
+      <c r="B50" s="8"/>
+      <c r="C50" s="8"/>
+      <c r="D50" s="8"/>
+      <c r="E50" s="8"/>
+      <c r="F50" s="8"/>
+      <c r="G50" s="8"/>
     </row>
     <row r="51" spans="1:7">
-      <c r="A51" s="7"/>
-      <c r="B51" s="7"/>
-      <c r="C51" s="7"/>
-      <c r="D51" s="7"/>
-      <c r="E51" s="7"/>
-      <c r="F51" s="7"/>
-      <c r="G51" s="7"/>
+      <c r="A51" s="8"/>
+      <c r="B51" s="8"/>
+      <c r="C51" s="8"/>
+      <c r="D51" s="8"/>
+      <c r="E51" s="8"/>
+      <c r="F51" s="8"/>
+      <c r="G51" s="8"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -2077,7 +2081,9 @@
         <v>50</v>
       </c>
       <c r="E2" s="4"/>
-      <c r="F2" s="2"/>
+      <c r="F2" s="5">
+        <v>46304</v>
+      </c>
     </row>
     <row r="3" ht="64" customHeight="1" spans="1:6">
       <c r="A3" s="2" t="s">
@@ -2093,9 +2099,11 @@
         <v>52</v>
       </c>
       <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-    </row>
-    <row r="4" ht="44" customHeight="1" spans="1:6">
+      <c r="F3" s="5">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="4" ht="67" customHeight="1" spans="1:6">
       <c r="A4" s="2" t="s">
         <v>19</v>
       </c>
@@ -2109,9 +2117,11 @@
         <v>54</v>
       </c>
       <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-    </row>
-    <row r="5" ht="45" customHeight="1" spans="1:6">
+      <c r="F4" s="5">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="5" ht="62" customHeight="1" spans="1:6">
       <c r="A5" s="2" t="s">
         <v>25</v>
       </c>
@@ -2125,9 +2135,11 @@
         <v>56</v>
       </c>
       <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-    </row>
-    <row r="6" ht="45" customHeight="1" spans="1:6">
+      <c r="F5" s="5">
+        <v>46304</v>
+      </c>
+    </row>
+    <row r="6" ht="65" customHeight="1" spans="1:6">
       <c r="A6" s="2" t="s">
         <v>29</v>
       </c>
@@ -2141,7 +2153,9 @@
         <v>57</v>
       </c>
       <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
+      <c r="F6" s="5">
+        <v>46304</v>
+      </c>
     </row>
     <row r="7" ht="74" customHeight="1" spans="1:6">
       <c r="A7" s="2" t="s">
@@ -2157,9 +2171,11 @@
         <v>59</v>
       </c>
       <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-    </row>
-    <row r="8" ht="42.75" spans="1:6">
+      <c r="F7" s="5">
+        <v>46305</v>
+      </c>
+    </row>
+    <row r="8" ht="59" customHeight="1" spans="1:6">
       <c r="A8" s="2" t="s">
         <v>39</v>
       </c>
@@ -2173,7 +2189,9 @@
         <v>61</v>
       </c>
       <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
+      <c r="F8" s="5">
+        <v>46305</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>